<commit_message>
updates metadata, addresses issue 7
</commit_message>
<xml_diff>
--- a/data-raw/metadata/yuba_adult_metadata.xlsx
+++ b/data-raw/metadata/yuba_adult_metadata.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Badhia\Documents\git\jpe-yuba-adult-edi\data-raw\metadata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6049EB-FA41-49BE-AD7A-FA4F4B358A07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{611CA883-8798-4818-894C-A7FC77D9116C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3530" yWindow="1040" windowWidth="19200" windowHeight="11170" firstSheet="4" activeTab="9" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-75" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="dataset" sheetId="1" r:id="rId1"/>
@@ -293,9 +293,6 @@
     <t>Yuba Water Agency</t>
   </si>
   <si>
-    <t>HDR, Inc.</t>
-  </si>
-  <si>
     <t>Yuba River Chinook Upstream Passage</t>
   </si>
   <si>
@@ -306,6 +303,9 @@
   </si>
   <si>
     <t>Jason</t>
+  </si>
+  <si>
+    <t>RBI</t>
   </si>
 </sst>
 </file>
@@ -712,7 +712,7 @@
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>3</v>
@@ -16822,7 +16822,7 @@
         <v>52</v>
       </c>
       <c r="E2" s="17" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="F2" s="18"/>
     </row>
@@ -16855,7 +16855,7 @@
         <v>56</v>
       </c>
       <c r="D4" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>53</v>
@@ -16864,7 +16864,7 @@
     </row>
     <row r="5" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B5" s="17" t="s">
         <v>59</v>
@@ -16873,7 +16873,7 @@
         <v>60</v>
       </c>
       <c r="D5" s="17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>53</v>
@@ -19896,10 +19896,10 @@
     </row>
     <row r="2" spans="1:2" ht="15.5" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.35"/>
@@ -50142,7 +50142,7 @@
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B2" s="16">
         <v>-121.51359600000001</v>

</xml_diff>